<commit_message>
feat(upload): implement document upload functionality in TerminalRestauranteShell
- Added a new feature to upload documents (PDF/images) in the TerminalRestauranteShell, enhancing user interaction.
- Integrated the upload functionality with the existing presenter to handle document processing and feedback.
- Updated UI components to include an upload button for document import, improving the overall user experience.

This update enriches the terminal's capabilities by allowing users to import relevant documents directly from the interface.
</commit_message>
<xml_diff>
--- a/docs/añadidos manual/registro desayuno.xlsx
+++ b/docs/añadidos manual/registro desayuno.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\HOTEL\REGISTRO DESAYUNO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\HOTEL\BM V.2\docs\añadidos manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550E276A-54A3-4D07-A2F4-6E8E7D811642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5B4DBD-D271-4D0F-9BE1-327716119077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="10" xr2:uid="{E9E04712-666D-44F1-AA33-F29703BA28A6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="17" xr2:uid="{E9E04712-666D-44F1-AA33-F29703BA28A6}"/>
   </bookViews>
   <sheets>
     <sheet name="01 " sheetId="1" r:id="rId1"/>
@@ -24,6 +24,13 @@
     <sheet name="09" sheetId="9" r:id="rId9"/>
     <sheet name="10" sheetId="10" r:id="rId10"/>
     <sheet name="11" sheetId="11" r:id="rId11"/>
+    <sheet name="13" sheetId="17" r:id="rId12"/>
+    <sheet name="14" sheetId="12" r:id="rId13"/>
+    <sheet name="15" sheetId="13" r:id="rId14"/>
+    <sheet name="16" sheetId="14" r:id="rId15"/>
+    <sheet name="17" sheetId="15" r:id="rId16"/>
+    <sheet name="18" sheetId="16" r:id="rId17"/>
+    <sheet name="19" sheetId="18" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="386">
   <si>
     <t>2 HUEVOS COCIDOS</t>
   </si>
@@ -835,6 +842,378 @@
   </si>
   <si>
     <t>DESAYUO NGLES SIN TOMATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TOSTADA DEL DIA SIN TOMATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOSTADA DEL DIA </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TORTILLA JAMON Y CEBOLLA </t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO, AGUACATE Y SALMON</t>
+  </si>
+  <si>
+    <t>X2 TORTILLA JAMON Y QUESO</t>
+  </si>
+  <si>
+    <t>SANDWICH DE LA CASA SIN QUESO</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHE, TOMATE, SALCHICA</t>
+  </si>
+  <si>
+    <t>DESAYUNA INGLES SIN ALUBIAS SIN HASHBROWN</t>
+  </si>
+  <si>
+    <t>X2 SANDWICH DE LA CASA</t>
+  </si>
+  <si>
+    <t>TORTILLA, TOMATE Y HASHBROWN</t>
+  </si>
+  <si>
+    <t>TOSTADA CHAMPI CON 2 HUEVO POCHE</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTOS, BACON Y ALUBIAS</t>
+  </si>
+  <si>
+    <t>X3 HUEVO REVUELTO</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON Y QUESO CON PAN SIN GLUTEN</t>
+  </si>
+  <si>
+    <t>2 HUEVO COCIDOS 2 BACON</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO CON TOSTADA</t>
+  </si>
+  <si>
+    <t>TOSTADA FRANBCESA</t>
+  </si>
+  <si>
+    <t>SANDWICH MIXTO CON HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>2 HUEVOS POCHADO CON SALCHICHA, BACON Y TOMATE</t>
+  </si>
+  <si>
+    <t>SANDWICH SOLO QUESO</t>
+  </si>
+  <si>
+    <t>TORTILLA CON QUESO</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO Y TOMATE</t>
+  </si>
+  <si>
+    <t>TORTILLA CON BACON Y TOMATE</t>
+  </si>
+  <si>
+    <t>SANDWICH CON JAMON Y QUESO</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO</t>
+  </si>
+  <si>
+    <t>TOSTADA DEL DIA X2</t>
+  </si>
+  <si>
+    <t>TORTILLA CON CHAMPI Y TOSTADA</t>
+  </si>
+  <si>
+    <t>TORTILLA CON JAMON Y QUESO Y PAN INTEGRAL</t>
+  </si>
+  <si>
+    <t>TORTILLA CON QUESO, TOMATE Y TOMATE Y CHAMPI</t>
+  </si>
+  <si>
+    <t>SANDWICH CON JAMON Y QUESO Y CHAMPI</t>
+  </si>
+  <si>
+    <t>2 HUEVOS POCHADO, TOSTADA, SALCHICHA Y HASHBROWN</t>
+  </si>
+  <si>
+    <t>HUEVO FRITO, 3 BACON, 2 PAN Y ALUBIAS</t>
+  </si>
+  <si>
+    <t>2 TOSTADAS DEL DIA</t>
+  </si>
+  <si>
+    <t>3 HUEVOS POCHADO Y 1 SANDWICH MIXTO</t>
+  </si>
+  <si>
+    <t>1 TORTILLA DE 3 HUEVOS Y TOMATE CHERRY</t>
+  </si>
+  <si>
+    <t>1 TORTILLA CON HASHBROWN Y TOMATE</t>
+  </si>
+  <si>
+    <t>1 TORTILLA CONM JAMON Y QUESO Y PAN SIN GLUTEN</t>
+  </si>
+  <si>
+    <t>2 HUEVOS Y 2 BACON</t>
+  </si>
+  <si>
+    <t>HUEVO</t>
+  </si>
+  <si>
+    <t>2 HUEVOS POCHADO, PAN, SALCHICHA, BACON Y TOMATE</t>
+  </si>
+  <si>
+    <t>TOSTADA DEL DIA Y HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>TOSTADA CHAMPI CON BACON</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO Y ESPINACAS</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO Y PAN MARRON</t>
+  </si>
+  <si>
+    <t>TORTILLA CHAMPIÑONES Y PAN</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON Y QUESO PAN SIN GLUTEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 HUEVOS  </t>
+  </si>
+  <si>
+    <t>BACON SALCHICHA Y HUEVO FRITO</t>
+  </si>
+  <si>
+    <t>TORTILLA QUESO Y JAMON X 2</t>
+  </si>
+  <si>
+    <t>TOSTADA DEL DIA Y 2 KIWI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TORTILLA JAMON Y QUESO   </t>
+  </si>
+  <si>
+    <t>TORTILLA QUESO Y CHAMPI</t>
+  </si>
+  <si>
+    <t>PAN MARRON</t>
+  </si>
+  <si>
+    <t>PAN SIN GLUTEN+</t>
+  </si>
+  <si>
+    <t>SALCHICHA Y BACON</t>
+  </si>
+  <si>
+    <t>TORTILLA X2</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO,. TOMATE CHERRY Y HASHBROWN</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO Y TOMATE CHERRY</t>
+  </si>
+  <si>
+    <t>SANDWICH VEGETAL EN PAN MARRON Y TOMATE</t>
+  </si>
+  <si>
+    <t>3 HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>TORTILLA CON ESPINACA Y QUESO</t>
+  </si>
+  <si>
+    <t>SANDWICH MIXTO Y HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>JAMON SERRANO Y QUESO X2</t>
+  </si>
+  <si>
+    <t>SANDWICH VEGETAL EN PAN MARRON</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON, PIMIENTO Y QUESO</t>
+  </si>
+  <si>
+    <t>PAN SIN GLUTEN, SANDWICH DE LA CASA Y UN HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>HUEVO POCHE</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHE Y BACON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TORTILLA 2 HAHSBROWN Y 2 TOMATE </t>
+  </si>
+  <si>
+    <t>HUEVO POCHE Y 2 TOMATE Y AGUACTAE</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO, TOMATE Y AGUACATE</t>
+  </si>
+  <si>
+    <t>HUEVO POCHE TOMATE Y AGUACATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANDWICH VEGETAL   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TORTILLA QUESO, CHAMPI, BACON </t>
+  </si>
+  <si>
+    <t>DESAYUNO INMGLES</t>
+  </si>
+  <si>
+    <t>2 HUEVO PCOHE</t>
+  </si>
+  <si>
+    <t>TORTILLA CHAMPI Y PAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 HUEVO POCHE  </t>
+  </si>
+  <si>
+    <t>TORTILLA QUESO Y ESPINACAS</t>
+  </si>
+  <si>
+    <t>TOSTDA FRANCESA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TORTILLA   </t>
+  </si>
+  <si>
+    <t>TORTILLA Y CHAMPI</t>
+  </si>
+  <si>
+    <t>2 HUEVO DURO</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHE</t>
+  </si>
+  <si>
+    <t>TORTILLA TOMATE Y HASHBROWN</t>
+  </si>
+  <si>
+    <t>HUEVO FRITO 2 TOMATE</t>
+  </si>
+  <si>
+    <t>2 HUEVO FRITO</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO Y TOSTADA MAROON</t>
+  </si>
+  <si>
+    <t>TORTILLA QUESO Y CHAMPI Y BACON</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO Y PAN INTEGRAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 HUEVO POCHADO Y TOSTADA </t>
+  </si>
+  <si>
+    <t>2 HUEVOS</t>
+  </si>
+  <si>
+    <t>HUEVO POCHADO</t>
+  </si>
+  <si>
+    <t>2 huevos</t>
+  </si>
+  <si>
+    <t>SANDWICH VEGETAL 2 HASHBROWN</t>
+  </si>
+  <si>
+    <t>2 TOMATE</t>
+  </si>
+  <si>
+    <t>HUEVO POCHADO X2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOMATE </t>
+  </si>
+  <si>
+    <t>2 HUEVOSHUEVO REVUELTOS</t>
+  </si>
+  <si>
+    <t>SANDWICH SOLO QUYESO</t>
+  </si>
+  <si>
+    <t>HUEVO FRITO BACON Y AGUACTAE</t>
+  </si>
+  <si>
+    <t>TORTILLA ESPINACAS BACON Y TOMATE</t>
+  </si>
+  <si>
+    <t>TORTILLA CHAMPIÑONES QUESO Y SALCHICHA</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTOS BACON Y JUYDIAS</t>
+  </si>
+  <si>
+    <t>DESAYUNO INGLES X2</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO, HUEVO FRITO Y 5 BACON</t>
+  </si>
+  <si>
+    <t>2 POCHADO PAN BACON SALCHICHA TOMATE</t>
+  </si>
+  <si>
+    <t>TORTILLA CHAMPI QUESO TOMATE</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON QUESO PAN SIN GLUTEN</t>
+  </si>
+  <si>
+    <t>2 HUEVOS 2 BACON</t>
+  </si>
+  <si>
+    <t>POCHADO BACON TOMATE</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON QUESO CHAMPI PIMIENTO</t>
+  </si>
+  <si>
+    <t>TOSTADA DIA X2</t>
+  </si>
+  <si>
+    <t>SANDWICH DE LA CASA X2</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO 3 HUEVOS</t>
+  </si>
+  <si>
+    <t>HUEVO POCHE X2</t>
+  </si>
+  <si>
+    <t>HUEVO POCHE X3 PAN INTEGRAÑ</t>
+  </si>
+  <si>
+    <t>TORTILLA JAMON Y QUESO Y BACON</t>
+  </si>
+  <si>
+    <t>HUEVO REVUELTO Y `PAN</t>
+  </si>
+  <si>
+    <t>HUEVO POCHE 2 TOMATE</t>
+  </si>
+  <si>
+    <t>HUEVO RITO DOS TOMATES</t>
+  </si>
+  <si>
+    <t>TORTILA 2 TOMATE Y HASBROWN</t>
+  </si>
+  <si>
+    <t>2 HUEVO POCHADO Y SALCHICHA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAN SIN GLUTEN </t>
   </si>
 </sst>
 </file>
@@ -1207,162 +1586,162 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6F81DEE-1C9F-4058-B786-3CC90A88D80A}">
   <dimension ref="A2:A32"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.73046875" customWidth="1"/>
+    <col min="1" max="1" width="48.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>24</v>
       </c>
@@ -1375,162 +1754,162 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81647A7E-19A1-42EC-B247-63BD95F57E86}">
   <dimension ref="A1:A31"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.33203125" customWidth="1"/>
+    <col min="1" max="1" width="45.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>243</v>
       </c>
@@ -1543,169 +1922,1170 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B61253-490D-4341-A170-2B5D3DCCD74E}">
   <dimension ref="A1:A32"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.73046875" customWidth="1"/>
+    <col min="1" max="1" width="61.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C65EF8F-C5A3-488A-8563-A21517FBAE6E}">
+  <dimension ref="A1:A23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>371</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4C66513-8B40-4ED5-9E71-9CCA90087E39}">
+  <dimension ref="A1:A24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="109.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>280</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD11DED5-519F-4FD1-BA67-710CD18DFB88}">
+  <dimension ref="A1:A27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="53.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28B6A011-D65D-44DF-8452-1627F04F034E}">
+  <dimension ref="A1:A29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="83" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>323</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2361CBDA-6FF2-4A6D-AE12-91D4E756594F}">
+  <dimension ref="A1:A29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="116.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73264D59-6A8C-4F02-AB83-C3AA212F9C66}">
+  <dimension ref="A1:A24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="86.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E477BF-6827-44DE-AC55-272CB041932D}">
+  <dimension ref="A1:A26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>354</v>
       </c>
     </row>
   </sheetData>
@@ -1716,147 +3096,147 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56ACA687-D633-4892-B088-06F8194CCBD0}">
   <dimension ref="A1:A28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="73.06640625" customWidth="1"/>
+    <col min="1" max="1" width="73" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>46</v>
       </c>
@@ -1869,162 +3249,162 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6F0B3F0-BF3F-4F43-8C15-E3C96784F23D}">
   <dimension ref="A1:A31"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.86328125" customWidth="1"/>
+    <col min="1" max="1" width="40.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>70</v>
       </c>
@@ -2037,212 +3417,212 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B48079D8-6716-4C25-A6A9-78BEB682B66B}">
   <dimension ref="A1:A41"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1328125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>101</v>
       </c>
@@ -2255,202 +3635,202 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEBBD19E-46E2-4F5C-BA2B-5E198D4C8B6C}">
   <dimension ref="A1:A39"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.796875" customWidth="1"/>
+    <col min="1" max="1" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>127</v>
       </c>
@@ -2463,182 +3843,182 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D9800B1-5AE0-4AAD-B88F-D97E359F850D}">
   <dimension ref="A1:A35"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.19921875" customWidth="1"/>
+    <col min="1" max="1" width="44.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>27</v>
       </c>
@@ -2651,172 +4031,172 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF08B95-EBED-4AF4-B9A7-40357F31E0EA}">
   <dimension ref="A1:A33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51.1328125" customWidth="1"/>
+    <col min="1" max="1" width="51.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>177</v>
       </c>
@@ -2829,192 +4209,192 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7306DD-1AEC-47A3-981A-96B092DDD14C}">
   <dimension ref="A1:A37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.796875" customWidth="1"/>
+    <col min="1" max="1" width="59.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>198</v>
       </c>
@@ -3027,167 +4407,167 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B44E941-5B88-4851-901C-F4CBE8567AAD}">
   <dimension ref="A1:A32"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.9296875" customWidth="1"/>
+    <col min="1" max="1" width="56" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>74</v>
       </c>

</xml_diff>